<commit_message>
S.no correction in LCSC BOM
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/LCSC-BOM.xlsx
+++ b/Deliverables/BOM/LCSC-BOM.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\JohnWollam-LCDProject\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\JohnWollam-LCDProject\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49863034-2F07-4634-B50F-B40940A55763}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D4F0E50A-C57A-4E56-80D6-C3E94E5D1AEE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -137,7 +136,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -684,7 +683,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2990240D-2E4D-4C3B-B27C-98B62FAFA8BB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -971,7 +970,7 @@
     </row>
     <row r="27" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="12">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>25</v>
@@ -982,7 +981,7 @@
     </row>
     <row r="28" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="12">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>26</v>
@@ -993,7 +992,7 @@
     </row>
     <row r="29" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="12">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>27</v>
@@ -1004,7 +1003,7 @@
     </row>
     <row r="30" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="12">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>28</v>
@@ -1015,7 +1014,7 @@
     </row>
     <row r="31" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="12">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>29</v>
@@ -1026,7 +1025,7 @@
     </row>
     <row r="32" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="12">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C32" s="17" t="s">
         <v>30</v>

</xml_diff>